<commit_message>
add CI for Python 3.11 through 3.14
</commit_message>
<xml_diff>
--- a/tests/data/test_data_standard.xlsx
+++ b/tests/data/test_data_standard.xlsx
@@ -413,91 +413,133 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
-        <v>72</v>
-      </c>
-      <c r="B1" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="C1" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="D1" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F1" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G1" t="n">
-        <v>4.5</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SiO2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Al2O3</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>FeOt</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CaO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MgO</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Na2O</t>
+        </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Sample1</t>
+          <t>K2O</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>68.5</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sample1</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>15.8</v>
+        <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>4.2</v>
+        <v>14.2</v>
       </c>
       <c r="D2" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="E2" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="F2" t="n">
-        <v>3.8</v>
+        <v>0.8</v>
       </c>
       <c r="G2" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Sample2</t>
-        </is>
+        <v>3.2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sample2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sample3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>76.2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C4" t="n">
         <v>12.5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D4" t="n">
         <v>2.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E4" t="n">
         <v>1.2</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F4" t="n">
         <v>0.5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G4" t="n">
         <v>3.6</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H4" t="n">
         <v>5.2</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Sample3</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[codex] add CI for Python 3.11 through 3.14 (#16)
* add CI for Python 3.11 through 3.14

* install linux qt runtime deps in ci
</commit_message>
<xml_diff>
--- a/tests/data/test_data_standard.xlsx
+++ b/tests/data/test_data_standard.xlsx
@@ -413,91 +413,133 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
-        <v>72</v>
-      </c>
-      <c r="B1" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="C1" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="D1" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F1" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G1" t="n">
-        <v>4.5</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SiO2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Al2O3</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>FeOt</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CaO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MgO</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Na2O</t>
+        </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Sample1</t>
+          <t>K2O</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>68.5</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sample1</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>15.8</v>
+        <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>4.2</v>
+        <v>14.2</v>
       </c>
       <c r="D2" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="E2" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="F2" t="n">
-        <v>3.8</v>
+        <v>0.8</v>
       </c>
       <c r="G2" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Sample2</t>
-        </is>
+        <v>3.2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sample2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sample3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>76.2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C4" t="n">
         <v>12.5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D4" t="n">
         <v>2.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E4" t="n">
         <v>1.2</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F4" t="n">
         <v>0.5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G4" t="n">
         <v>3.6</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H4" t="n">
         <v>5.2</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Sample3</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>